<commit_message>
Actualización de Matriz de Trazabilidad
</commit_message>
<xml_diff>
--- a/Avance de Proyecto/PMOinformatica Plantilla de matriz de trazabilidad de requisitos.xls.xlsx
+++ b/Avance de Proyecto/PMOinformatica Plantilla de matriz de trazabilidad de requisitos.xls.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c84f6c42465ed23/Escritorio/MASTER/Universidad/9no Semestre/Comunicacion de Datos/ProyIntComDat25B_3.1416chul-s/ProyIntComDat25B_3.1416chul-s/Avance de Proyecto/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lmeji\Desktop\MASTER\Universidad\9no Semestre\Comunicacion de Datos\ProyIntComDat25B_3.1416chul-s\ProyIntComDat25B_3.1416chul-s\Avance de Proyecto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="8_{E6591D62-A935-45D6-9911-A6F8A66ACAC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D765A1D-182A-48F4-B68B-AAFD4D01FCAB}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB930B3E-2DFD-45D3-845B-E8324E28810E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8595" yWindow="0" windowWidth="12000" windowHeight="10905" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="10455" windowHeight="10905" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plantilla de matriz requisitos" sheetId="1" r:id="rId1"/>
@@ -1177,7 +1177,7 @@
         <v>21</v>
       </c>
       <c r="F7" s="15">
-        <v>45930</v>
+        <v>45944</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>158</v>
@@ -1237,7 +1237,7 @@
         <v>21</v>
       </c>
       <c r="F8" s="15">
-        <v>45930</v>
+        <v>45944</v>
       </c>
       <c r="G8" s="8" t="s">
         <v>30</v>
@@ -1297,7 +1297,7 @@
         <v>37</v>
       </c>
       <c r="F9" s="15">
-        <v>45930</v>
+        <v>45944</v>
       </c>
       <c r="G9" s="8" t="s">
         <v>38</v>
@@ -1357,7 +1357,7 @@
         <v>37</v>
       </c>
       <c r="F10" s="15">
-        <v>45930</v>
+        <v>45961</v>
       </c>
       <c r="G10" s="8" t="s">
         <v>165</v>
@@ -1417,7 +1417,7 @@
         <v>21</v>
       </c>
       <c r="F11" s="15">
-        <v>45930</v>
+        <v>45940</v>
       </c>
       <c r="G11" s="12" t="s">
         <v>42</v>
@@ -1477,7 +1477,7 @@
         <v>37</v>
       </c>
       <c r="F12" s="15">
-        <v>45930</v>
+        <v>45940</v>
       </c>
       <c r="G12" s="12" t="s">
         <v>50</v>
@@ -1537,7 +1537,7 @@
         <v>37</v>
       </c>
       <c r="F13" s="15">
-        <v>45930</v>
+        <v>45944</v>
       </c>
       <c r="G13" s="8" t="s">
         <v>58</v>
@@ -1597,7 +1597,7 @@
         <v>37</v>
       </c>
       <c r="F14" s="15">
-        <v>45931</v>
+        <v>45955</v>
       </c>
       <c r="G14" s="8" t="s">
         <v>65</v>
@@ -1657,7 +1657,7 @@
         <v>37</v>
       </c>
       <c r="F15" s="15">
-        <v>45931</v>
+        <v>45955</v>
       </c>
       <c r="G15" s="8" t="s">
         <v>65</v>
@@ -1717,7 +1717,7 @@
         <v>37</v>
       </c>
       <c r="F16" s="15">
-        <v>45931</v>
+        <v>45957</v>
       </c>
       <c r="G16" s="8" t="s">
         <v>65</v>
@@ -1777,7 +1777,7 @@
         <v>37</v>
       </c>
       <c r="F17" s="15">
-        <v>45982</v>
+        <v>45961</v>
       </c>
       <c r="G17" s="8" t="s">
         <v>65</v>
@@ -1837,7 +1837,7 @@
         <v>37</v>
       </c>
       <c r="F18" s="15">
-        <v>45984</v>
+        <v>45962</v>
       </c>
       <c r="G18" s="8" t="s">
         <v>74</v>
@@ -1897,7 +1897,7 @@
         <v>37</v>
       </c>
       <c r="F19" s="15">
-        <v>45990</v>
+        <v>45966</v>
       </c>
       <c r="G19" s="8" t="s">
         <v>81</v>
@@ -1957,7 +1957,7 @@
         <v>37</v>
       </c>
       <c r="F20" s="15">
-        <v>45990</v>
+        <v>45968</v>
       </c>
       <c r="G20" s="8" t="s">
         <v>89</v>
@@ -2017,7 +2017,7 @@
         <v>37</v>
       </c>
       <c r="F21" s="15">
-        <v>45949</v>
+        <v>45971</v>
       </c>
       <c r="G21" s="8" t="s">
         <v>94</v>
@@ -2077,7 +2077,7 @@
         <v>37</v>
       </c>
       <c r="F22" s="15">
-        <v>46003</v>
+        <v>45976</v>
       </c>
       <c r="G22" s="8" t="s">
         <v>101</v>
@@ -2137,7 +2137,7 @@
         <v>37</v>
       </c>
       <c r="F23" s="15">
-        <v>46002</v>
+        <v>45981</v>
       </c>
       <c r="G23" s="8" t="s">
         <v>107</v>
@@ -2197,7 +2197,7 @@
         <v>37</v>
       </c>
       <c r="F24" s="15">
-        <v>46011</v>
+        <v>45989</v>
       </c>
       <c r="G24" s="8" t="s">
         <v>114</v>
@@ -2257,7 +2257,7 @@
         <v>37</v>
       </c>
       <c r="F25" s="15">
-        <v>46023</v>
+        <v>45994</v>
       </c>
       <c r="G25" s="8" t="s">
         <v>123</v>
@@ -2317,7 +2317,7 @@
         <v>37</v>
       </c>
       <c r="F26" s="15">
-        <v>46052</v>
+        <v>45996</v>
       </c>
       <c r="G26" s="8" t="s">
         <v>132</v>
@@ -57757,6 +57757,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101004C1A3113D649624F9135CDBD3D69C302" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="13ffc8dcfefe0bebfe1d287b721fe34d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="6af09f24-5ef0-42a5-957c-ff861d9f3bca" xmlns:ns4="0fa9766c-9bcd-4ad8-8425-98b74b0d2252" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="df4ecb7d677b47b7113d60f963805797" ns3:_="" ns4:_="">
     <xsd:import namespace="6af09f24-5ef0-42a5-957c-ff861d9f3bca"/>
@@ -57983,15 +57992,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E1DE7B6-29CE-4FAD-801A-1BB807154730}">
   <ds:schemaRefs>
@@ -58010,6 +58010,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12716809-A2C5-4BB3-BB0A-F0C3124F50CB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EED8B2CD-5E4B-4E79-A91C-8550F2629E73}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -58026,12 +58034,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12716809-A2C5-4BB3-BB0A-F0C3124F50CB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>